<commit_message>
Enhance report pipeline with CLI options, date parsing improvements, and test coverage
</commit_message>
<xml_diff>
--- a/archive/2026-09-04/before_process/dong gop cua vingroup/Dong gop cua vingroup_update 040926.xlsx
+++ b/archive/2026-09-04/before_process/dong gop cua vingroup/Dong gop cua vingroup_update 040926.xlsx
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.0;\-#,##0;\-"/>
     <numFmt numFmtId="165" formatCode="#,##0.0_ ;\-#,##0.0\ "/>
     <numFmt numFmtId="166" formatCode="mm/dd/yyyy"/>
@@ -23,7 +23,6 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="#,##0.0_);\(#,##0.0\)"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -5575,7 +5574,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -5622,7 +5621,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -8316,7 +8315,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -8376,7 +8375,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>

</xml_diff>